<commit_message>
update Inventory to v2_3; Bugfix in GNFR C
</commit_message>
<xml_diff>
--- a/output/2019/sector_totals_2019.xlsx
+++ b/output/2019/sector_totals_2019.xlsx
@@ -492,22 +492,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1796.316270913122</v>
+        <v>1796.316268090944</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>683.1349231141756</v>
+        <v>674.2759232188134</v>
       </c>
       <c r="E3" t="n">
-        <v>394.9544215286256</v>
+        <v>396.0761462369327</v>
       </c>
       <c r="F3" t="n">
-        <v>79.37230812425607</v>
+        <v>80.25878484434527</v>
       </c>
       <c r="G3" t="n">
-        <v>4.449361053106772</v>
+        <v>4.415037341564879</v>
       </c>
     </row>
     <row r="4">
@@ -817,22 +817,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6714.272751141971</v>
+        <v>6714.272748319794</v>
       </c>
       <c r="C16" t="n">
         <v>534.0051445905361</v>
       </c>
       <c r="D16" t="n">
-        <v>6367.318488511512</v>
+        <v>6358.45948861615</v>
       </c>
       <c r="E16" t="n">
-        <v>7910.739008973328</v>
+        <v>7911.860733681636</v>
       </c>
       <c r="F16" t="n">
-        <v>4493.607804500877</v>
+        <v>4494.494281220967</v>
       </c>
       <c r="G16" t="n">
-        <v>49.32103049837363</v>
+        <v>49.28670678683174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates for v2_3 upload to ICOS CP
</commit_message>
<xml_diff>
--- a/output/2019/sector_totals_2019.xlsx
+++ b/output/2019/sector_totals_2019.xlsx
@@ -492,22 +492,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1796.316268090944</v>
+        <v>1905.031022805004</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>674.2759232188134</v>
+        <v>752.6597374617714</v>
       </c>
       <c r="E3" t="n">
-        <v>396.0761462369327</v>
+        <v>2128.523411618597</v>
       </c>
       <c r="F3" t="n">
-        <v>80.25878484434527</v>
+        <v>188.6936922353829</v>
       </c>
       <c r="G3" t="n">
-        <v>4.415037341564879</v>
+        <v>83.44932914660238</v>
       </c>
     </row>
     <row r="4">
@@ -817,22 +817,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6714.272748319794</v>
+        <v>6822.987503033853</v>
       </c>
       <c r="C16" t="n">
         <v>534.0051445905361</v>
       </c>
       <c r="D16" t="n">
-        <v>6358.45948861615</v>
+        <v>6436.843302859108</v>
       </c>
       <c r="E16" t="n">
-        <v>7911.860733681636</v>
+        <v>9644.307999063298</v>
       </c>
       <c r="F16" t="n">
-        <v>4494.494281220967</v>
+        <v>4602.929188612005</v>
       </c>
       <c r="G16" t="n">
-        <v>49.28670678683174</v>
+        <v>128.3209985918692</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
gnfr c wood combustion moved to co2 bio
</commit_message>
<xml_diff>
--- a/output/2019/sector_totals_2019.xlsx
+++ b/output/2019/sector_totals_2019.xlsx
@@ -492,22 +492,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1905.031022805004</v>
+        <v>1793.566742622751</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>111.464280182253</v>
       </c>
       <c r="D3" t="n">
         <v>752.6597374617714</v>
       </c>
       <c r="E3" t="n">
-        <v>2128.523411618597</v>
+        <v>2128.523411618596</v>
       </c>
       <c r="F3" t="n">
         <v>188.6936922353829</v>
       </c>
       <c r="G3" t="n">
-        <v>83.44932914660238</v>
+        <v>83.44932914660237</v>
       </c>
     </row>
     <row r="4">
@@ -817,10 +817,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6822.987503033853</v>
+        <v>6711.5232228516</v>
       </c>
       <c r="C16" t="n">
-        <v>534.0051445905361</v>
+        <v>645.4694247727891</v>
       </c>
       <c r="D16" t="n">
         <v>6436.843302859108</v>

</xml_diff>

<commit_message>
update to inventory v2.4
</commit_message>
<xml_diff>
--- a/output/2019/sector_totals_2019.xlsx
+++ b/output/2019/sector_totals_2019.xlsx
@@ -470,7 +470,7 @@
         <v>3033.4</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>294.998</v>
       </c>
       <c r="D2" t="n">
         <v>1989.8</v>
@@ -492,22 +492,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1793.566742622751</v>
+        <v>1919.662801140333</v>
       </c>
       <c r="C3" t="n">
-        <v>111.464280182253</v>
+        <v>126.0960585175821</v>
       </c>
       <c r="D3" t="n">
-        <v>752.6597374617714</v>
+        <v>762.8902477764684</v>
       </c>
       <c r="E3" t="n">
-        <v>2128.523411618596</v>
+        <v>2355.954181245558</v>
       </c>
       <c r="F3" t="n">
-        <v>188.6936922353829</v>
+        <v>203.1706032992287</v>
       </c>
       <c r="G3" t="n">
-        <v>83.44932914660237</v>
+        <v>93.82387591726278</v>
       </c>
     </row>
     <row r="4">
@@ -817,22 +817,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6711.5232228516</v>
+        <v>6837.619281369181</v>
       </c>
       <c r="C16" t="n">
-        <v>645.4694247727891</v>
+        <v>955.0992031081182</v>
       </c>
       <c r="D16" t="n">
-        <v>6436.843302859108</v>
+        <v>6447.073813173805</v>
       </c>
       <c r="E16" t="n">
-        <v>9644.307999063298</v>
+        <v>9871.738768690258</v>
       </c>
       <c r="F16" t="n">
-        <v>4602.929188612005</v>
+        <v>4617.40609967585</v>
       </c>
       <c r="G16" t="n">
-        <v>128.3209985918692</v>
+        <v>138.6955453625296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>